<commit_message>
change in json schema and added resume pdf download button
</commit_message>
<xml_diff>
--- a/job_applications.xlsx
+++ b/job_applications.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Applications'!$A$1:$AB$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Applications'!$A$1:$AB$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -907,8 +907,226 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>APP-20260117122114</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Applied Scientist - AI/ML, Decision Intelligence Team</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Seattle, WA (On-site)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Company Website</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>full-time</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>84.2%</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>83.1%</t>
+        </is>
+      </c>
+      <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr"/>
+      <c r="U6" s="3" t="inlineStr"/>
+      <c r="V6" s="3" t="inlineStr"/>
+      <c r="W6" s="4" t="inlineStr"/>
+      <c r="X6" s="4" t="inlineStr"/>
+      <c r="Y6" s="3" t="inlineStr"/>
+      <c r="Z6" s="4" t="inlineStr"/>
+      <c r="AA6" s="4" t="inlineStr">
+        <is>
+          <t>Python, Machine Learning, Deep Learning, PyTorch, TensorFlow</t>
+        </is>
+      </c>
+      <c r="AB6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>APP-20260117123711</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AI Solutions Developer</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Company Website</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>full-time</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>84.2%</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>90.1%</t>
+        </is>
+      </c>
+      <c r="U7" s="5" t="inlineStr"/>
+      <c r="V7" s="5" t="inlineStr"/>
+      <c r="Y7" s="5" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Python, Machine Learning Fundamentals, Natural Language Processing, Generative AI, Problem-solving</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>APP-20260117125215</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Klaviyo</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>AI Platform Engineer</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Boston, MA (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Company Website</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>full-time</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>84.2%</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr"/>
+      <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="inlineStr"/>
+      <c r="U8" s="3" t="inlineStr"/>
+      <c r="V8" s="3" t="inlineStr"/>
+      <c r="W8" s="4" t="inlineStr"/>
+      <c r="X8" s="4" t="inlineStr"/>
+      <c r="Y8" s="3" t="inlineStr"/>
+      <c r="Z8" s="4" t="inlineStr"/>
+      <c r="AA8" s="4" t="inlineStr">
+        <is>
+          <t>Backend Systems, Distributed Systems, Python, Generative AI, Agentic AI</t>
+        </is>
+      </c>
+      <c r="AB8" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB5"/>
+  <autoFilter ref="A1:AB8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>